<commit_message>
added pregnancy obj 1.3 and 1.4. Clean up of other scripts before second release
</commit_message>
<xml_diff>
--- a/DEVELOPMENT/ADEPTOBJ1_scripts/definitions/bridge/ADEPT_O1_BRIDGE_19Mayo25.xlsx
+++ b/DEVELOPMENT/ADEPTOBJ1_scripts/definitions/bridge/ADEPT_O1_BRIDGE_19Mayo25.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mgamb\Documents\GitHub\ADEPT_obj1\DEVELOPMENT\ADEPTOBJ1_scripts\definitions\bridge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE6ED66-FF49-4C28-9085-43594B9CDF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFADD1DB-3464-445A-AFCB-758CB0889C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="2424" windowWidth="21600" windowHeight="11232" xr2:uid="{2506CD93-0285-9E44-BBDD-A2C4E77A0341}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2506CD93-0285-9E44-BBDD-A2C4E77A0341}"/>
   </bookViews>
   <sheets>
     <sheet name="OBJ1" sheetId="5" r:id="rId1"/>
@@ -1777,7 +1777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1809,6 +1809,7 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2129,7 +2130,7 @@
   <dimension ref="A1:K179"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.09765625" customWidth="1"/>
+    <col min="1" max="1" width="36.796875" customWidth="1"/>
     <col min="2" max="2" width="14.59765625" customWidth="1"/>
     <col min="3" max="3" width="13.19921875" customWidth="1"/>
     <col min="4" max="4" width="9"/>
@@ -2212,17 +2213,15 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A3" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="9"/>
       <c r="C3" t="b">
         <v>0</v>
       </c>
       <c r="D3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -2231,24 +2230,21 @@
         <v>0</v>
       </c>
       <c r="G3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
       </c>
-      <c r="J3" t="b">
-        <v>0</v>
-      </c>
       <c r="K3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -2278,12 +2274,12 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -2313,12 +2309,12 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -2348,12 +2344,12 @@
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -2383,53 +2379,53 @@
         <v>0</v>
       </c>
       <c r="K7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" t="b">
         <v>0</v>
@@ -2453,37 +2449,42 @@
         <v>1</v>
       </c>
       <c r="K9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="9"/>
-      <c r="C10" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" t="b">
-        <v>0</v>
-      </c>
-      <c r="I10" t="b">
-        <v>0</v>
-      </c>
-      <c r="K10" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
@@ -2523,13 +2524,10 @@
     </row>
     <row r="12" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="9" t="b">
-        <v>0</v>
+        <v>359</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
       </c>
       <c r="D12" t="b">
         <v>0</v>
@@ -2541,30 +2539,24 @@
         <v>0</v>
       </c>
       <c r="G12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
       </c>
-      <c r="J12" t="b">
-        <v>1</v>
-      </c>
       <c r="K12" t="s">
-        <v>16</v>
+        <v>360</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>313</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="9" t="b">
-        <v>0</v>
+      <c r="A13" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
       </c>
       <c r="D13" t="b">
         <v>0</v>
@@ -2576,55 +2568,51 @@
         <v>0</v>
       </c>
       <c r="G13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" t="b">
         <v>1</v>
       </c>
-      <c r="J13" t="b">
-        <v>1</v>
-      </c>
       <c r="K13" t="s">
-        <v>314</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>127</v>
+        <v>319</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="D14" s="9" t="b">
+      <c r="D14" t="b">
         <v>0</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
       </c>
       <c r="F14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="H14" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="I14" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9" t="s">
-        <v>128</v>
+        <v>1</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>6</v>
@@ -2654,12 +2642,12 @@
         <v>1</v>
       </c>
       <c r="K15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>297</v>
+        <v>313</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>6</v>
@@ -2689,20 +2677,18 @@
         <v>1</v>
       </c>
       <c r="K16" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>6</v>
-      </c>
+      <c r="A17" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="9"/>
       <c r="C17" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="9" t="b">
         <v>0</v>
       </c>
       <c r="E17" t="b">
@@ -2711,31 +2697,29 @@
       <c r="F17" t="b">
         <v>0</v>
       </c>
-      <c r="G17" t="b">
-        <v>0</v>
-      </c>
-      <c r="H17" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17" t="b">
-        <v>1</v>
-      </c>
-      <c r="J17" t="b">
-        <v>1</v>
-      </c>
-      <c r="K17" t="s">
-        <v>20</v>
+      <c r="G17" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C18" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="b">
         <v>0</v>
@@ -2759,12 +2743,12 @@
         <v>1</v>
       </c>
       <c r="K18" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>197</v>
+      <c r="A19" t="s">
+        <v>297</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>6</v>
@@ -2794,12 +2778,12 @@
         <v>1</v>
       </c>
       <c r="K19" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>6</v>
@@ -2829,18 +2813,18 @@
         <v>1</v>
       </c>
       <c r="K20" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>331</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C21" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="b">
         <v>0</v>
@@ -2864,14 +2848,15 @@
         <v>1</v>
       </c>
       <c r="K21" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
-        <v>359</v>
-      </c>
-      <c r="C22" t="b">
+        <v>191</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D22" t="b">
@@ -2892,16 +2877,20 @@
       <c r="I22" t="b">
         <v>1</v>
       </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
       <c r="K22" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
-        <v>357</v>
-      </c>
-      <c r="C23" t="b">
-        <v>1</v>
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>317</v>
+      </c>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9" t="b">
+        <v>0</v>
       </c>
       <c r="D23" t="b">
         <v>0</v>
@@ -2910,7 +2899,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="b">
         <v>1</v>
@@ -2922,14 +2911,16 @@
         <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>358</v>
+        <v>318</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>319</v>
-      </c>
-      <c r="B24" s="9"/>
+      <c r="A24" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C24" s="9" t="b">
         <v>0</v>
       </c>
@@ -2940,30 +2931,33 @@
         <v>0</v>
       </c>
       <c r="F24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="b">
         <v>1</v>
       </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
       <c r="K24" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C25" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" t="b">
         <v>0</v>
@@ -2987,70 +2981,77 @@
         <v>1</v>
       </c>
       <c r="K25" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>331</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
+      </c>
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" t="b">
+        <v>0</v>
+      </c>
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" t="b">
+        <v>0</v>
+      </c>
+      <c r="G27" t="b">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="b">
+        <v>1</v>
+      </c>
+      <c r="K27" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D26" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" t="b">
-        <v>0</v>
-      </c>
-      <c r="F26" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" t="b">
-        <v>1</v>
-      </c>
-      <c r="H26" t="b">
-        <v>0</v>
-      </c>
-      <c r="I26" t="b">
-        <v>1</v>
-      </c>
-      <c r="J26" t="b">
-        <v>1</v>
-      </c>
-      <c r="K26" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>317</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="D27" t="b">
-        <v>0</v>
-      </c>
-      <c r="E27" t="b">
-        <v>0</v>
-      </c>
-      <c r="F27" t="b">
-        <v>1</v>
-      </c>
-      <c r="G27" t="b">
-        <v>1</v>
-      </c>
-      <c r="H27" t="b">
-        <v>0</v>
-      </c>
-      <c r="I27" t="b">
-        <v>1</v>
-      </c>
-      <c r="K27" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
@@ -3158,7 +3159,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>37</v>
       </c>
@@ -3193,7 +3194,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>61</v>
       </c>
@@ -3228,7 +3229,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>63</v>
       </c>
@@ -3264,10 +3265,12 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>337</v>
-      </c>
-      <c r="B34" s="9"/>
+      <c r="A34" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C34" s="9" t="b">
         <v>0</v>
       </c>
@@ -3278,30 +3281,33 @@
         <v>0</v>
       </c>
       <c r="F34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" t="b">
         <v>1</v>
       </c>
+      <c r="J34" t="b">
+        <v>1</v>
+      </c>
       <c r="K34" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B35" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C35" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" t="b">
         <v>0</v>
@@ -3325,12 +3331,12 @@
         <v>1</v>
       </c>
       <c r="K35" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>6</v>
@@ -3360,18 +3366,18 @@
         <v>1</v>
       </c>
       <c r="K36" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
-        <v>69</v>
+      <c r="A37" t="s">
+        <v>59</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C37" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" t="b">
         <v>0</v>
@@ -3392,15 +3398,15 @@
         <v>1</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>59</v>
+      <c r="A38" s="9" t="s">
+        <v>233</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>6</v>
@@ -3430,12 +3436,12 @@
         <v>0</v>
       </c>
       <c r="K38" t="s">
-        <v>60</v>
+        <v>234</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="B39" s="9"/>
       <c r="C39" s="9" t="b">
@@ -3460,14 +3466,16 @@
         <v>1</v>
       </c>
       <c r="K39" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>321</v>
-      </c>
-      <c r="B40" s="9"/>
+      <c r="A40" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C40" s="9" t="b">
         <v>0</v>
       </c>
@@ -3478,24 +3486,27 @@
         <v>0</v>
       </c>
       <c r="F40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" t="b">
         <v>1</v>
       </c>
+      <c r="J40" t="b">
+        <v>1</v>
+      </c>
       <c r="K40" t="s">
-        <v>322</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="9" t="s">
-        <v>233</v>
+      <c r="A41" t="s">
+        <v>329</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>6</v>
@@ -3522,21 +3533,21 @@
         <v>1</v>
       </c>
       <c r="J41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C42" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" t="b">
         <v>0</v>
@@ -3560,18 +3571,18 @@
         <v>1</v>
       </c>
       <c r="K42" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>329</v>
-      </c>
-      <c r="B43" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="B43" t="s">
         <v>6</v>
       </c>
-      <c r="C43" s="9" t="b">
-        <v>0</v>
+      <c r="C43" t="b">
+        <v>1</v>
       </c>
       <c r="D43" t="b">
         <v>0</v>
@@ -3595,14 +3606,16 @@
         <v>1</v>
       </c>
       <c r="K43" t="s">
-        <v>330</v>
+        <v>356</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>311</v>
-      </c>
-      <c r="B44" s="9"/>
+      <c r="A44" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C44" s="9" t="b">
         <v>0</v>
       </c>
@@ -3613,30 +3626,33 @@
         <v>0</v>
       </c>
       <c r="F44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" t="b">
         <v>1</v>
       </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
       <c r="K44" t="s">
-        <v>312</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B45" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C45" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" t="b">
         <v>0</v>
@@ -3660,20 +3676,20 @@
         <v>1</v>
       </c>
       <c r="K45" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
-        <v>355</v>
-      </c>
-      <c r="B46" t="s">
+        <v>125</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C46" t="b">
-        <v>1</v>
-      </c>
-      <c r="D46" t="b">
+      <c r="C46" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D46" s="9" t="b">
         <v>0</v>
       </c>
       <c r="E46" t="b">
@@ -3682,29 +3698,27 @@
       <c r="F46" t="b">
         <v>0</v>
       </c>
-      <c r="G46" t="b">
-        <v>0</v>
-      </c>
-      <c r="H46" t="b">
-        <v>1</v>
-      </c>
-      <c r="I46" t="b">
-        <v>1</v>
-      </c>
-      <c r="J46" t="b">
-        <v>1</v>
-      </c>
-      <c r="K46" t="s">
-        <v>356</v>
+      <c r="G46" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H46" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J46" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K46" s="9" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B47" s="9" t="s">
-        <v>6</v>
-      </c>
+      <c r="A47" t="s">
+        <v>323</v>
+      </c>
+      <c r="B47" s="9"/>
       <c r="C47" s="9" t="b">
         <v>0</v>
       </c>
@@ -3715,27 +3729,24 @@
         <v>0</v>
       </c>
       <c r="F47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
-      <c r="J47" t="b">
-        <v>1</v>
-      </c>
       <c r="K47" t="s">
-        <v>78</v>
+        <v>324</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>79</v>
+      <c r="A48" t="s">
+        <v>295</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>6</v>
@@ -3765,12 +3776,12 @@
         <v>1</v>
       </c>
       <c r="K48" t="s">
-        <v>80</v>
+        <v>296</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="9" t="s">
-        <v>125</v>
+        <v>85</v>
       </c>
       <c r="B49" s="9" t="s">
         <v>6</v>
@@ -3778,7 +3789,7 @@
       <c r="C49" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="D49" s="9" t="b">
+      <c r="D49" t="b">
         <v>0</v>
       </c>
       <c r="E49" t="b">
@@ -3787,25 +3798,25 @@
       <c r="F49" t="b">
         <v>0</v>
       </c>
-      <c r="G49" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="H49" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="I49" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="J49" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="K49" s="9" t="s">
-        <v>126</v>
+      <c r="G49" t="b">
+        <v>0</v>
+      </c>
+      <c r="H49" t="b">
+        <v>1</v>
+      </c>
+      <c r="I49" t="b">
+        <v>1</v>
+      </c>
+      <c r="J49" t="b">
+        <v>1</v>
+      </c>
+      <c r="K49" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>295</v>
+      <c r="A50" s="9" t="s">
+        <v>87</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>6</v>
@@ -3835,18 +3846,18 @@
         <v>1</v>
       </c>
       <c r="K50" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C51" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D51" t="b">
         <v>0</v>
@@ -3870,16 +3881,14 @@
         <v>1</v>
       </c>
       <c r="K51" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>6</v>
-      </c>
+      <c r="A52" t="s">
+        <v>321</v>
+      </c>
+      <c r="B52" s="9"/>
       <c r="C52" s="9" t="b">
         <v>0</v>
       </c>
@@ -3890,27 +3899,24 @@
         <v>0</v>
       </c>
       <c r="F52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
-      <c r="J52" t="b">
-        <v>1</v>
-      </c>
       <c r="K52" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>6</v>
@@ -3940,12 +3946,12 @@
         <v>1</v>
       </c>
       <c r="K53" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B54" s="9" t="s">
         <v>6</v>
@@ -3975,12 +3981,12 @@
         <v>1</v>
       </c>
       <c r="K54" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>6</v>
@@ -4010,12 +4016,12 @@
         <v>1</v>
       </c>
       <c r="K55" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B56" s="9" t="s">
         <v>6</v>
@@ -4045,14 +4051,16 @@
         <v>1</v>
       </c>
       <c r="K56" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B57" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C57" s="9" t="b">
         <v>1</v>
       </c>
@@ -4066,24 +4074,24 @@
         <v>0</v>
       </c>
       <c r="G57" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K57" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B58" s="9" t="s">
         <v>6</v>
@@ -4113,18 +4121,18 @@
         <v>1</v>
       </c>
       <c r="K58" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B59" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C59" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D59" t="b">
         <v>0</v>
@@ -4148,18 +4156,18 @@
         <v>1</v>
       </c>
       <c r="K59" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B60" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C60" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D60" t="b">
         <v>0</v>
@@ -4183,14 +4191,16 @@
         <v>1</v>
       </c>
       <c r="K60" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="B61" s="9"/>
+      <c r="A61" t="s">
+        <v>285</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C61" s="9" t="b">
         <v>0</v>
       </c>
@@ -4201,26 +4211,31 @@
         <v>0</v>
       </c>
       <c r="F61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
+      <c r="J61" t="b">
+        <v>1</v>
+      </c>
       <c r="K61" t="s">
-        <v>186</v>
+        <v>286</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>327</v>
-      </c>
-      <c r="B62" s="9"/>
+      <c r="A62" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>6</v>
+      </c>
       <c r="C62" s="9" t="b">
         <v>0</v>
       </c>
@@ -4231,24 +4246,27 @@
         <v>0</v>
       </c>
       <c r="F62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" t="b">
         <v>1</v>
       </c>
+      <c r="J62" t="b">
+        <v>1</v>
+      </c>
       <c r="K62" t="s">
-        <v>328</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="9" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B63" s="9" t="s">
         <v>6</v>
@@ -4278,18 +4296,18 @@
         <v>1</v>
       </c>
       <c r="K63" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B64" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C64" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D64" t="b">
         <v>0</v>
@@ -4313,15 +4331,17 @@
         <v>1</v>
       </c>
       <c r="K64" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>353</v>
-      </c>
-      <c r="B65" s="9"/>
-      <c r="C65" t="b">
+      <c r="A65" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C65" s="9" t="b">
         <v>0</v>
       </c>
       <c r="D65" t="b">
@@ -4331,30 +4351,33 @@
         <v>0</v>
       </c>
       <c r="F65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
+      <c r="J65" t="b">
+        <v>1</v>
+      </c>
       <c r="K65" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>285</v>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A66" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="B66" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C66" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D66" t="b">
         <v>0</v>
@@ -4378,18 +4401,16 @@
         <v>1</v>
       </c>
       <c r="K66" t="s">
-        <v>286</v>
+        <v>118</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>6</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="B67" s="9"/>
       <c r="C67" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D67" t="b">
         <v>0</v>
@@ -4401,24 +4422,24 @@
         <v>0</v>
       </c>
       <c r="G67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K67" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="9" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B68" s="9" t="s">
         <v>6</v>
@@ -4448,12 +4469,12 @@
         <v>1</v>
       </c>
       <c r="K68" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="9" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B69" s="9" t="s">
         <v>6</v>
@@ -4483,12 +4504,12 @@
         <v>1</v>
       </c>
       <c r="K69" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="9" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="B70" s="9" t="s">
         <v>6</v>
@@ -4518,18 +4539,18 @@
         <v>1</v>
       </c>
       <c r="K70" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
     </row>
     <row r="71" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="9" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="B71" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C71" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D71" t="b">
         <v>0</v>
@@ -4553,12 +4574,12 @@
         <v>1</v>
       </c>
       <c r="K71" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="72" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="9" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="B72" s="9" t="s">
         <v>6</v>
@@ -4588,18 +4609,18 @@
         <v>1</v>
       </c>
       <c r="K72" t="s">
-        <v>122</v>
+        <v>142</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="9" t="s">
-        <v>123</v>
+        <v>35</v>
       </c>
       <c r="B73" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C73" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D73" t="b">
         <v>0</v>
@@ -4620,20 +4641,20 @@
         <v>1</v>
       </c>
       <c r="J73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="s">
-        <v>124</v>
+        <v>36</v>
       </c>
     </row>
     <row r="74" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="B74" s="9" t="s">
+      <c r="A74" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="B74" t="s">
         <v>6</v>
       </c>
-      <c r="C74" s="9" t="b">
+      <c r="C74" t="b">
         <v>0</v>
       </c>
       <c r="D74" t="b">
@@ -4658,18 +4679,18 @@
         <v>1</v>
       </c>
       <c r="K74" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="9" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="B75" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C75" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D75" t="b">
         <v>0</v>
@@ -4693,18 +4714,18 @@
         <v>1</v>
       </c>
       <c r="K75" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="9" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B76" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C76" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D76" t="b">
         <v>0</v>
@@ -4728,18 +4749,18 @@
         <v>1</v>
       </c>
       <c r="K76" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="9" t="s">
-        <v>35</v>
+        <v>149</v>
       </c>
       <c r="B77" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C77" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D77" t="b">
         <v>0</v>
@@ -4760,20 +4781,20 @@
         <v>1</v>
       </c>
       <c r="J77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K77" t="s">
-        <v>36</v>
+        <v>150</v>
       </c>
     </row>
     <row r="78" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="13" t="s">
-        <v>361</v>
-      </c>
-      <c r="B78" t="s">
+      <c r="A78" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B78" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C78" t="b">
+      <c r="C78" s="9" t="b">
         <v>0</v>
       </c>
       <c r="D78" t="b">
@@ -4798,18 +4819,18 @@
         <v>1</v>
       </c>
       <c r="K78" t="s">
-        <v>362</v>
+        <v>40</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B79" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C79" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D79" t="b">
         <v>0</v>
@@ -4833,18 +4854,18 @@
         <v>1</v>
       </c>
       <c r="K79" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="9" t="s">
-        <v>147</v>
+      <c r="A80" s="14" t="s">
+        <v>151</v>
       </c>
       <c r="B80" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C80" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D80" t="b">
         <v>0</v>
@@ -4868,18 +4889,18 @@
         <v>1</v>
       </c>
       <c r="K80" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="9" t="s">
-        <v>149</v>
+      <c r="A81" t="s">
+        <v>307</v>
       </c>
       <c r="B81" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C81" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D81" t="b">
         <v>0</v>
@@ -4903,19 +4924,21 @@
         <v>1</v>
       </c>
       <c r="K81" t="s">
-        <v>150</v>
+        <v>308</v>
       </c>
     </row>
     <row r="82" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>351</v>
-      </c>
-      <c r="B82" s="14"/>
-      <c r="C82" t="b">
+      <c r="A82" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B82" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C82" s="9" t="b">
         <v>0</v>
       </c>
       <c r="D82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -4924,27 +4947,30 @@
         <v>0</v>
       </c>
       <c r="G82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="b">
         <v>0</v>
       </c>
       <c r="K82" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A83" s="9" t="s">
-        <v>39</v>
+        <v>155</v>
       </c>
       <c r="B83" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C83" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D83" t="b">
         <v>0</v>
@@ -4968,12 +4994,12 @@
         <v>1</v>
       </c>
       <c r="K83" t="s">
-        <v>40</v>
+        <v>156</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="9" t="s">
-        <v>143</v>
+      <c r="A84" t="s">
+        <v>315</v>
       </c>
       <c r="B84" s="9" t="s">
         <v>6</v>
@@ -5003,12 +5029,12 @@
         <v>1</v>
       </c>
       <c r="K84" t="s">
-        <v>144</v>
+        <v>316</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="14" t="s">
-        <v>151</v>
+      <c r="A85" t="s">
+        <v>343</v>
       </c>
       <c r="B85" s="9" t="s">
         <v>6</v>
@@ -5035,15 +5061,15 @@
         <v>1</v>
       </c>
       <c r="J85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K85" t="s">
-        <v>152</v>
+        <v>344</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>307</v>
+        <v>157</v>
       </c>
       <c r="B86" s="9" t="s">
         <v>6</v>
@@ -5073,18 +5099,18 @@
         <v>1</v>
       </c>
       <c r="K86" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="9" t="s">
-        <v>153</v>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>159</v>
       </c>
       <c r="B87" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C87" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D87" t="b">
         <v>0</v>
@@ -5105,15 +5131,15 @@
         <v>1</v>
       </c>
       <c r="J87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K87" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="9" t="s">
-        <v>155</v>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>161</v>
       </c>
       <c r="B88" s="9" t="s">
         <v>6</v>
@@ -5143,18 +5169,18 @@
         <v>1</v>
       </c>
       <c r="K88" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>315</v>
+        <v>163</v>
       </c>
       <c r="B89" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C89" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D89" t="b">
         <v>0</v>
@@ -5178,18 +5204,18 @@
         <v>1</v>
       </c>
       <c r="K89" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>343</v>
+        <v>165</v>
       </c>
       <c r="B90" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C90" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D90" t="b">
         <v>0</v>
@@ -5210,15 +5236,15 @@
         <v>1</v>
       </c>
       <c r="J90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K90" t="s">
-        <v>344</v>
+        <v>166</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>157</v>
+      <c r="A91" s="14" t="s">
+        <v>167</v>
       </c>
       <c r="B91" s="9" t="s">
         <v>6</v>
@@ -5248,12 +5274,12 @@
         <v>1</v>
       </c>
       <c r="K91" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="B92" s="9" t="s">
         <v>6</v>
@@ -5283,18 +5309,16 @@
         <v>1</v>
       </c>
       <c r="K92" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>161</v>
-      </c>
-      <c r="B93" s="9" t="s">
-        <v>6</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="B93" s="9"/>
       <c r="C93" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D93" t="b">
         <v>0</v>
@@ -5303,33 +5327,30 @@
         <v>0</v>
       </c>
       <c r="F93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I93" t="b">
         <v>1</v>
       </c>
-      <c r="J93" t="b">
-        <v>1</v>
-      </c>
       <c r="K93" t="s">
-        <v>162</v>
+        <v>312</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>163</v>
+      <c r="A94" s="14" t="s">
+        <v>173</v>
       </c>
       <c r="B94" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C94" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D94" t="b">
         <v>0</v>
@@ -5353,12 +5374,12 @@
         <v>1</v>
       </c>
       <c r="K94" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>165</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A95" s="9" t="s">
+        <v>175</v>
       </c>
       <c r="B95" s="9" t="s">
         <v>6</v>
@@ -5388,12 +5409,12 @@
         <v>1</v>
       </c>
       <c r="K95" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="14" t="s">
-        <v>167</v>
+      <c r="A96" s="9" t="s">
+        <v>177</v>
       </c>
       <c r="B96" s="9" t="s">
         <v>6</v>
@@ -5423,18 +5444,18 @@
         <v>1</v>
       </c>
       <c r="K96" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>169</v>
+        <v>345</v>
       </c>
       <c r="B97" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C97" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D97" t="b">
         <v>0</v>
@@ -5458,12 +5479,12 @@
         <v>1</v>
       </c>
       <c r="K97" t="s">
-        <v>170</v>
+        <v>346</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="14" t="s">
-        <v>173</v>
+      <c r="A98" s="9" t="s">
+        <v>179</v>
       </c>
       <c r="B98" s="9" t="s">
         <v>6</v>
@@ -5493,18 +5514,18 @@
         <v>1</v>
       </c>
       <c r="K98" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="9" t="s">
-        <v>175</v>
+      <c r="A99" t="s">
+        <v>299</v>
       </c>
       <c r="B99" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C99" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D99" t="b">
         <v>0</v>
@@ -5528,12 +5549,12 @@
         <v>1</v>
       </c>
       <c r="K99" t="s">
-        <v>176</v>
+        <v>300</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="9" t="s">
-        <v>177</v>
+      <c r="A100" t="s">
+        <v>333</v>
       </c>
       <c r="B100" s="9" t="s">
         <v>6</v>
@@ -5563,16 +5584,14 @@
         <v>1</v>
       </c>
       <c r="K100" t="s">
-        <v>178</v>
+        <v>334</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
-        <v>345</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>6</v>
-      </c>
+      <c r="A101" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B101" s="9"/>
       <c r="C101" s="9" t="b">
         <v>0</v>
       </c>
@@ -5583,27 +5602,24 @@
         <v>0</v>
       </c>
       <c r="F101" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G101" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H101" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I101" t="b">
         <v>1</v>
       </c>
-      <c r="J101" t="b">
-        <v>1</v>
-      </c>
       <c r="K101" t="s">
-        <v>346</v>
+        <v>186</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="9" t="s">
-        <v>179</v>
+      <c r="A102" t="s">
+        <v>301</v>
       </c>
       <c r="B102" s="9" t="s">
         <v>6</v>
@@ -5633,12 +5649,12 @@
         <v>1</v>
       </c>
       <c r="K102" t="s">
-        <v>180</v>
+        <v>302</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B103" s="9" t="s">
         <v>6</v>
@@ -5668,12 +5684,12 @@
         <v>1</v>
       </c>
       <c r="K103" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
-        <v>333</v>
+      <c r="A104" s="9" t="s">
+        <v>183</v>
       </c>
       <c r="B104" s="9" t="s">
         <v>6</v>
@@ -5703,12 +5719,12 @@
         <v>1</v>
       </c>
       <c r="K104" t="s">
-        <v>334</v>
+        <v>184</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>301</v>
+      <c r="A105" s="9" t="s">
+        <v>187</v>
       </c>
       <c r="B105" s="9" t="s">
         <v>6</v>
@@ -5735,15 +5751,15 @@
         <v>1</v>
       </c>
       <c r="J105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K105" t="s">
-        <v>302</v>
+        <v>188</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
-        <v>305</v>
+      <c r="A106" s="9" t="s">
+        <v>189</v>
       </c>
       <c r="B106" s="9" t="s">
         <v>6</v>
@@ -5773,12 +5789,12 @@
         <v>1</v>
       </c>
       <c r="K106" t="s">
-        <v>306</v>
+        <v>190</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="9" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="B107" s="9" t="s">
         <v>6</v>
@@ -5805,21 +5821,21 @@
         <v>1</v>
       </c>
       <c r="J107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K107" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A108" s="9" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B108" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C108" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D108" t="b">
         <v>0</v>
@@ -5840,15 +5856,15 @@
         <v>1</v>
       </c>
       <c r="J108" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K108" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="9" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="B109" s="9" t="s">
         <v>6</v>
@@ -5878,18 +5894,18 @@
         <v>1</v>
       </c>
       <c r="K109" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="110" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A110" s="9" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B110" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C110" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D110" t="b">
         <v>0</v>
@@ -5910,21 +5926,21 @@
         <v>1</v>
       </c>
       <c r="J110" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K110" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="9" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B111" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C111" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D111" t="b">
         <v>0</v>
@@ -5948,18 +5964,18 @@
         <v>1</v>
       </c>
       <c r="K111" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="112" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A112" s="9" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B112" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C112" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D112" t="b">
         <v>0</v>
@@ -5983,12 +5999,12 @@
         <v>1</v>
       </c>
       <c r="K112" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="113" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A113" s="9" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B113" s="9" t="s">
         <v>6</v>
@@ -6018,18 +6034,18 @@
         <v>1</v>
       </c>
       <c r="K113" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A114" s="9" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B114" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C114" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D114" t="b">
         <v>0</v>
@@ -6053,12 +6069,12 @@
         <v>1</v>
       </c>
       <c r="K114" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A115" s="9" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B115" s="9" t="s">
         <v>6</v>
@@ -6088,12 +6104,12 @@
         <v>1</v>
       </c>
       <c r="K115" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="116" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A116" s="9" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B116" s="9" t="s">
         <v>6</v>
@@ -6123,12 +6139,12 @@
         <v>1</v>
       </c>
       <c r="K116" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A117" s="9" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B117" s="9" t="s">
         <v>6</v>
@@ -6158,18 +6174,18 @@
         <v>1</v>
       </c>
       <c r="K117" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="9" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B118" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C118" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D118" t="b">
         <v>0</v>
@@ -6193,12 +6209,12 @@
         <v>1</v>
       </c>
       <c r="K118" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="119" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A119" s="9" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B119" s="9" t="s">
         <v>6</v>
@@ -6228,12 +6244,12 @@
         <v>1</v>
       </c>
       <c r="K119" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="120" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A120" s="9" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B120" s="9" t="s">
         <v>6</v>
@@ -6263,18 +6279,18 @@
         <v>1</v>
       </c>
       <c r="K120" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="9" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B121" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C121" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D121" t="b">
         <v>0</v>
@@ -6298,18 +6314,18 @@
         <v>1</v>
       </c>
       <c r="K121" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="9" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="B122" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C122" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D122" t="b">
         <v>0</v>
@@ -6333,18 +6349,18 @@
         <v>1</v>
       </c>
       <c r="K122" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="9" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B123" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C123" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D123" t="b">
         <v>0</v>
@@ -6368,18 +6384,16 @@
         <v>1</v>
       </c>
       <c r="K123" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="B124" s="9" t="s">
-        <v>6</v>
-      </c>
+      <c r="A124" t="s">
+        <v>327</v>
+      </c>
+      <c r="B124" s="9"/>
       <c r="C124" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D124" t="b">
         <v>0</v>
@@ -6388,33 +6402,30 @@
         <v>0</v>
       </c>
       <c r="F124" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G124" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H124" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I124" t="b">
         <v>1</v>
       </c>
-      <c r="J124" t="b">
-        <v>1</v>
-      </c>
       <c r="K124" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="125" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A125" s="9" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="B125" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C125" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D125" t="b">
         <v>0</v>
@@ -6438,12 +6449,12 @@
         <v>1</v>
       </c>
       <c r="K125" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="9" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="B126" s="9" t="s">
         <v>6</v>
@@ -6473,18 +6484,18 @@
         <v>1</v>
       </c>
       <c r="K126" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="9" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B127" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C127" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D127" t="b">
         <v>0</v>
@@ -6508,18 +6519,18 @@
         <v>1</v>
       </c>
       <c r="K127" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>243</v>
       </c>
       <c r="B128" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C128" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D128" t="b">
         <v>0</v>
@@ -6543,17 +6554,15 @@
         <v>1</v>
       </c>
       <c r="K128" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="B129" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C129" s="9" t="b">
+      <c r="A129" t="s">
+        <v>353</v>
+      </c>
+      <c r="B129" s="9"/>
+      <c r="C129" t="b">
         <v>0</v>
       </c>
       <c r="D129" t="b">
@@ -6563,33 +6572,30 @@
         <v>0</v>
       </c>
       <c r="F129" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G129" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I129" t="b">
         <v>1</v>
       </c>
-      <c r="J129" t="b">
-        <v>1</v>
-      </c>
       <c r="K129" t="s">
-        <v>242</v>
+        <v>354</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
-        <v>243</v>
+      <c r="A130" s="9" t="s">
+        <v>247</v>
       </c>
       <c r="B130" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C130" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D130" t="b">
         <v>0</v>
@@ -6613,12 +6619,12 @@
         <v>1</v>
       </c>
       <c r="K130" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="9" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B131" s="9" t="s">
         <v>6</v>
@@ -6648,18 +6654,18 @@
         <v>1</v>
       </c>
       <c r="K131" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="132" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A132" s="9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B132" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C132" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D132" t="b">
         <v>0</v>
@@ -6683,12 +6689,12 @@
         <v>1</v>
       </c>
       <c r="K132" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="133" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A133" s="9" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B133" s="9" t="s">
         <v>6</v>
@@ -6718,18 +6724,18 @@
         <v>1</v>
       </c>
       <c r="K133" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="9" t="s">
-        <v>255</v>
+      <c r="A134" t="s">
+        <v>287</v>
       </c>
       <c r="B134" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C134" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D134" t="b">
         <v>0</v>
@@ -6750,22 +6756,24 @@
         <v>1</v>
       </c>
       <c r="J134" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K134" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="135" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B135" s="9"/>
-      <c r="C135" t="b">
-        <v>0</v>
+        <v>257</v>
+      </c>
+      <c r="B135" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C135" s="9" t="b">
+        <v>1</v>
       </c>
       <c r="D135" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -6774,21 +6782,24 @@
         <v>0</v>
       </c>
       <c r="G135" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H135" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I135" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J135" t="b">
+        <v>1</v>
       </c>
       <c r="K135" t="s">
-        <v>26</v>
+        <v>258</v>
       </c>
     </row>
     <row r="136" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" t="s">
-        <v>287</v>
+      <c r="A136" s="9" t="s">
+        <v>137</v>
       </c>
       <c r="B136" s="9" t="s">
         <v>6</v>
@@ -6815,15 +6826,15 @@
         <v>1</v>
       </c>
       <c r="J136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K136" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="137" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="9" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B137" s="9" t="s">
         <v>6</v>
@@ -6853,19 +6864,21 @@
         <v>1</v>
       </c>
       <c r="K137" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="B138" s="10"/>
-      <c r="C138" t="b">
+      <c r="A138" t="s">
+        <v>335</v>
+      </c>
+      <c r="B138" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C138" s="9" t="b">
         <v>0</v>
       </c>
       <c r="D138" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -6874,27 +6887,30 @@
         <v>0</v>
       </c>
       <c r="G138" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H138" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I138" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J138" t="b">
+        <v>1</v>
       </c>
       <c r="K138" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="9" t="s">
-        <v>137</v>
+        <v>261</v>
       </c>
       <c r="B139" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C139" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D139" t="b">
         <v>0</v>
@@ -6918,12 +6934,12 @@
         <v>1</v>
       </c>
       <c r="K139" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="140" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="9" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B140" s="9" t="s">
         <v>6</v>
@@ -6953,18 +6969,18 @@
         <v>1</v>
       </c>
       <c r="K140" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="141" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" t="s">
-        <v>335</v>
+        <v>264</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="9" t="s">
+        <v>265</v>
       </c>
       <c r="B141" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C141" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D141" t="b">
         <v>0</v>
@@ -6988,18 +7004,18 @@
         <v>1</v>
       </c>
       <c r="K141" t="s">
-        <v>336</v>
+        <v>266</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="9" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B142" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C142" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D142" t="b">
         <v>0</v>
@@ -7023,18 +7039,18 @@
         <v>1</v>
       </c>
       <c r="K142" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="143" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="9" t="s">
-        <v>263</v>
+      <c r="A143" t="s">
+        <v>303</v>
       </c>
       <c r="B143" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C143" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D143" t="b">
         <v>0</v>
@@ -7058,12 +7074,12 @@
         <v>1</v>
       </c>
       <c r="K143" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="144" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="9" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B144" s="9" t="s">
         <v>6</v>
@@ -7093,12 +7109,12 @@
         <v>1</v>
       </c>
       <c r="K144" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="9" t="s">
-        <v>267</v>
+      <c r="A145" t="s">
+        <v>339</v>
       </c>
       <c r="B145" s="9" t="s">
         <v>6</v>
@@ -7128,12 +7144,12 @@
         <v>1</v>
       </c>
       <c r="K145" t="s">
-        <v>268</v>
+        <v>340</v>
       </c>
     </row>
     <row r="146" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>303</v>
+        <v>341</v>
       </c>
       <c r="B146" s="9" t="s">
         <v>6</v>
@@ -7163,18 +7179,18 @@
         <v>1</v>
       </c>
       <c r="K146" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
     </row>
     <row r="147" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B147" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C147" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D147" t="b">
         <v>0</v>
@@ -7198,18 +7214,18 @@
         <v>1</v>
       </c>
       <c r="K147" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="148" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" t="s">
-        <v>339</v>
+        <v>272</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="9" t="s">
+        <v>273</v>
       </c>
       <c r="B148" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C148" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D148" t="b">
         <v>0</v>
@@ -7233,17 +7249,17 @@
         <v>1</v>
       </c>
       <c r="K148" t="s">
-        <v>340</v>
+        <v>274</v>
       </c>
     </row>
     <row r="149" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>341</v>
-      </c>
-      <c r="B149" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C149" s="9" t="b">
+        <v>347</v>
+      </c>
+      <c r="B149" t="s">
+        <v>9</v>
+      </c>
+      <c r="C149" t="b">
         <v>0</v>
       </c>
       <c r="D149" t="b">
@@ -7262,27 +7278,25 @@
         <v>1</v>
       </c>
       <c r="I149" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J149" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K149" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
     </row>
     <row r="150" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="B150" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C150" s="9" t="b">
+      <c r="A150" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="B150" s="14"/>
+      <c r="C150" t="b">
         <v>0</v>
       </c>
       <c r="D150" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -7291,30 +7305,27 @@
         <v>0</v>
       </c>
       <c r="G150" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H150" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I150" t="b">
-        <v>1</v>
-      </c>
-      <c r="J150" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K150" t="s">
-        <v>272</v>
+        <v>352</v>
       </c>
     </row>
     <row r="151" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="B151" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C151" s="9" t="b">
-        <v>1</v>
+      <c r="A151" t="s">
+        <v>349</v>
+      </c>
+      <c r="B151" t="s">
+        <v>9</v>
+      </c>
+      <c r="C151" t="b">
+        <v>0</v>
       </c>
       <c r="D151" t="b">
         <v>0</v>
@@ -7332,20 +7343,20 @@
         <v>1</v>
       </c>
       <c r="I151" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J151" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K151" t="s">
-        <v>274</v>
+        <v>350</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" t="s">
-        <v>347</v>
-      </c>
-      <c r="B152" t="s">
+      <c r="A152" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B152" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C152" t="b">
@@ -7355,7 +7366,7 @@
         <v>0</v>
       </c>
       <c r="E152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F152" t="b">
         <v>0</v>
@@ -7364,7 +7375,7 @@
         <v>0</v>
       </c>
       <c r="H152" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I152" t="b">
         <v>0</v>
@@ -7373,14 +7384,14 @@
         <v>0</v>
       </c>
       <c r="K152" t="s">
-        <v>348</v>
+        <v>236</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" t="s">
-        <v>349</v>
-      </c>
-      <c r="B153" t="s">
+      <c r="A153" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B153" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C153" t="b">
@@ -7390,7 +7401,7 @@
         <v>0</v>
       </c>
       <c r="E153" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F153" t="b">
         <v>0</v>
@@ -7399,7 +7410,7 @@
         <v>0</v>
       </c>
       <c r="H153" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I153" t="b">
         <v>0</v>
@@ -7408,12 +7419,12 @@
         <v>0</v>
       </c>
       <c r="K153" t="s">
-        <v>350</v>
+        <v>130</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="9" t="s">
-        <v>235</v>
+      <c r="A154" s="19" t="s">
+        <v>23</v>
       </c>
       <c r="B154" s="9" t="s">
         <v>9</v>
@@ -7440,17 +7451,17 @@
         <v>0</v>
       </c>
       <c r="J154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K154" t="s">
-        <v>236</v>
+        <v>24</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="B155" s="9" t="s">
+      <c r="A155" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="B155" t="s">
         <v>9</v>
       </c>
       <c r="C155" t="b">
@@ -7478,12 +7489,12 @@
         <v>0</v>
       </c>
       <c r="K155" t="s">
-        <v>130</v>
+        <v>292</v>
       </c>
     </row>
     <row r="156" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="9" t="s">
-        <v>23</v>
+        <v>249</v>
       </c>
       <c r="B156" s="9" t="s">
         <v>9</v>
@@ -7492,10 +7503,10 @@
         <v>0</v>
       </c>
       <c r="D156" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E156" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F156" t="b">
         <v>0</v>
@@ -7510,17 +7521,17 @@
         <v>0</v>
       </c>
       <c r="J156" t="b">
-        <v>1</v>
-      </c>
-      <c r="K156" t="s">
-        <v>24</v>
+        <v>0</v>
+      </c>
+      <c r="K156" s="11" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="157" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" t="s">
-        <v>291</v>
-      </c>
-      <c r="B157" t="s">
+      <c r="A157" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="B157" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C157" t="b">
@@ -7548,12 +7559,12 @@
         <v>0</v>
       </c>
       <c r="K157" t="s">
-        <v>292</v>
+        <v>246</v>
       </c>
     </row>
     <row r="158" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="9" t="s">
-        <v>249</v>
+        <v>139</v>
       </c>
       <c r="B158" s="9" t="s">
         <v>9</v>
@@ -7582,15 +7593,15 @@
       <c r="J158" t="b">
         <v>0</v>
       </c>
-      <c r="K158" s="11" t="s">
-        <v>250</v>
+      <c r="K158" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="159" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="B159" s="9" t="s">
+      <c r="A159" t="s">
+        <v>277</v>
+      </c>
+      <c r="B159" t="s">
         <v>9</v>
       </c>
       <c r="C159" t="b">
@@ -7600,7 +7611,7 @@
         <v>0</v>
       </c>
       <c r="E159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F159" t="b">
         <v>0</v>
@@ -7609,7 +7620,7 @@
         <v>0</v>
       </c>
       <c r="H159" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I159" t="b">
         <v>0</v>
@@ -7618,51 +7629,46 @@
         <v>0</v>
       </c>
       <c r="K159" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
     </row>
     <row r="160" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="B160" s="9" t="s">
+      <c r="A160" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B160" s="9"/>
+      <c r="C160" t="b">
+        <v>0</v>
+      </c>
+      <c r="D160" t="b">
+        <v>1</v>
+      </c>
+      <c r="E160" t="b">
+        <v>0</v>
+      </c>
+      <c r="F160" t="b">
+        <v>0</v>
+      </c>
+      <c r="G160" t="b">
+        <v>1</v>
+      </c>
+      <c r="H160" t="b">
+        <v>0</v>
+      </c>
+      <c r="I160" t="b">
+        <v>0</v>
+      </c>
+      <c r="K160" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="161" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="B161" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C160" t="b">
-        <v>0</v>
-      </c>
-      <c r="D160" t="b">
-        <v>1</v>
-      </c>
-      <c r="E160" t="b">
-        <v>0</v>
-      </c>
-      <c r="F160" t="b">
-        <v>0</v>
-      </c>
-      <c r="G160" t="b">
-        <v>0</v>
-      </c>
-      <c r="H160" t="b">
-        <v>0</v>
-      </c>
-      <c r="I160" t="b">
-        <v>0</v>
-      </c>
-      <c r="J160" t="b">
-        <v>0</v>
-      </c>
-      <c r="K160" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="161" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" t="s">
-        <v>277</v>
-      </c>
-      <c r="B161" t="s">
-        <v>9</v>
-      </c>
       <c r="C161" t="b">
         <v>0</v>
       </c>
@@ -7670,7 +7676,7 @@
         <v>0</v>
       </c>
       <c r="E161" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F161" t="b">
         <v>0</v>
@@ -7679,7 +7685,7 @@
         <v>0</v>
       </c>
       <c r="H161" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I161" t="b">
         <v>0</v>
@@ -7688,12 +7694,12 @@
         <v>0</v>
       </c>
       <c r="K161" t="s">
-        <v>278</v>
+        <v>84</v>
       </c>
     </row>
     <row r="162" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" t="s">
-        <v>83</v>
+      <c r="A162" s="9" t="s">
+        <v>71</v>
       </c>
       <c r="B162" s="9" t="s">
         <v>9</v>
@@ -7705,7 +7711,7 @@
         <v>0</v>
       </c>
       <c r="E162" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F162" t="b">
         <v>0</v>
@@ -7714,7 +7720,7 @@
         <v>0</v>
       </c>
       <c r="H162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I162" t="b">
         <v>0</v>
@@ -7723,21 +7729,19 @@
         <v>0</v>
       </c>
       <c r="K162" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B163" s="9" t="s">
-        <v>9</v>
-      </c>
+      <c r="A163" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="B163" s="10"/>
       <c r="C163" t="b">
         <v>0</v>
       </c>
       <c r="D163" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -7746,23 +7750,20 @@
         <v>0</v>
       </c>
       <c r="G163" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H163" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I163" t="b">
         <v>0</v>
       </c>
-      <c r="J163" t="b">
-        <v>0</v>
-      </c>
       <c r="K163" t="s">
-        <v>72</v>
+        <v>276</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="9" t="s">
+      <c r="A164" s="19" t="s">
         <v>81</v>
       </c>
       <c r="B164" s="9" t="s">
@@ -7797,7 +7798,7 @@
       </c>
     </row>
     <row r="165" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="9" t="s">
+      <c r="A165" s="19" t="s">
         <v>91</v>
       </c>
       <c r="B165" s="9" t="s">
@@ -7867,7 +7868,7 @@
       </c>
     </row>
     <row r="167" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="9" t="s">
+      <c r="A167" s="19" t="s">
         <v>171</v>
       </c>
       <c r="B167" s="9" t="s">
@@ -8077,10 +8078,12 @@
       </c>
     </row>
     <row r="173" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" t="s">
-        <v>293</v>
-      </c>
-      <c r="B173" s="10"/>
+      <c r="A173" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B173" s="9" t="s">
+        <v>9</v>
+      </c>
       <c r="C173" t="b">
         <v>0</v>
       </c>
@@ -8088,27 +8091,30 @@
         <v>0</v>
       </c>
       <c r="E173" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F173" t="b">
         <v>0</v>
       </c>
       <c r="G173" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H173" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I173" t="b">
         <v>0</v>
       </c>
+      <c r="J173" t="b">
+        <v>0</v>
+      </c>
       <c r="K173" t="s">
-        <v>294</v>
+        <v>136</v>
       </c>
     </row>
     <row r="174" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="9" t="s">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="B174" s="9" t="s">
         <v>9</v>
@@ -8138,22 +8144,22 @@
         <v>0</v>
       </c>
       <c r="K174" t="s">
-        <v>136</v>
+        <v>182</v>
       </c>
     </row>
     <row r="175" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A175" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="B175" s="9"/>
+      <c r="A175" s="18" t="s">
+        <v>293</v>
+      </c>
+      <c r="B175" s="10"/>
       <c r="C175" t="b">
         <v>0</v>
       </c>
       <c r="D175" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E175" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F175" t="b">
         <v>0</v>
@@ -8168,12 +8174,12 @@
         <v>0</v>
       </c>
       <c r="K175" t="s">
-        <v>230</v>
+        <v>294</v>
       </c>
     </row>
     <row r="176" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="9" t="s">
-        <v>181</v>
+        <v>231</v>
       </c>
       <c r="B176" s="9" t="s">
         <v>9</v>
@@ -8203,21 +8209,19 @@
         <v>0</v>
       </c>
       <c r="K176" t="s">
-        <v>182</v>
+        <v>232</v>
       </c>
     </row>
     <row r="177" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A177" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="B177" s="9" t="s">
-        <v>9</v>
-      </c>
+      <c r="A177" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="B177" s="9"/>
       <c r="C177" t="b">
         <v>0</v>
       </c>
       <c r="D177" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -8226,19 +8230,16 @@
         <v>0</v>
       </c>
       <c r="G177" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H177" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I177" t="b">
         <v>0</v>
       </c>
-      <c r="J177" t="b">
-        <v>0</v>
-      </c>
       <c r="K177" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="178" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -8277,7 +8278,7 @@
       </c>
     </row>
     <row r="179" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A179" t="s">
+      <c r="A179" s="18" t="s">
         <v>289</v>
       </c>
       <c r="B179" t="s">
@@ -8313,10 +8314,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K179" xr:uid="{E0FDDF39-709C-C14C-B461-AFB2AA297754}">
-    <filterColumn colId="1">
-      <filters blank="1"/>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="TRUE"/>
+      </filters>
     </filterColumn>
-    <filterColumn colId="2">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="FALSE"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="7">
       <filters>
         <filter val="TRUE"/>
       </filters>

</xml_diff>